<commit_message>
fix bulk tenant draft contract import
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_tenant_draft_contracts.xlsx
+++ b/docs/SLMS2026_import_tenant_draft_contracts.xlsx
@@ -573,7 +573,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:S6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -610,24 +610,27 @@
         <v>Nơi cấp CCCD</v>
       </c>
       <c r="L1" t="str">
+        <v>Hộ khẩu thường trú</v>
+      </c>
+      <c r="M1" t="str">
         <v>Ngày vào ở</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Ngày kết thúc</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Giá thuê/tháng</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Số tháng cọc</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Tiền cọc</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Ngày đón khách dự kiến</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>SĐT quản lý đón khách</v>
       </c>
     </row>
@@ -666,24 +669,27 @@
         <v>CA TP. Hồ Chí Minh</v>
       </c>
       <c r="L2" t="str">
+        <v>123 Nguyễn Huệ, Q1, TP.HCM</v>
+      </c>
+      <c r="M2" t="str">
         <v>2026-08-01</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>2027-07-31</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>8000000</v>
       </c>
-      <c r="O2">
+      <c r="P2">
         <v>1</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>8000000</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="R2" t="str">
         <v>2026-08-01</v>
       </c>
-      <c r="R2" t="str">
+      <c r="S2" t="str">
         <v/>
       </c>
     </row>
@@ -722,24 +728,27 @@
         <v>CA Quận 1</v>
       </c>
       <c r="L3" t="str">
+        <v>45 Lê Lợi, Q1, TP.HCM</v>
+      </c>
+      <c r="M3" t="str">
         <v>01/09/2026</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>31/08/2027</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>9500000</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>2</v>
       </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
       <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
         <v>01/09/2026</v>
       </c>
-      <c r="R3" t="str">
+      <c r="S3" t="str">
         <v/>
       </c>
     </row>
@@ -778,24 +787,27 @@
         <v>CA Bình Thạnh</v>
       </c>
       <c r="L4" t="str">
+        <v>88 Phạm Văn Đồng, Bình Thạnh, TP.HCM</v>
+      </c>
+      <c r="M4" t="str">
         <v>2026-08-15</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>2027-08-14</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>4500000</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>1</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>4500000</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="R4" t="str">
         <v>2026-08-15</v>
       </c>
-      <c r="R4" t="str">
+      <c r="S4" t="str">
         <v/>
       </c>
     </row>
@@ -834,24 +846,27 @@
         <v>CA Gò Vấp</v>
       </c>
       <c r="L5" t="str">
+        <v>12 Quang Trung, Gò Vấp, TP.HCM</v>
+      </c>
+      <c r="M5" t="str">
         <v>2026-08-15</v>
       </c>
-      <c r="M5" t="str">
+      <c r="N5" t="str">
         <v>2027-02-14</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>4200000</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>1</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>4200000</v>
       </c>
-      <c r="Q5" t="str">
+      <c r="R5" t="str">
         <v>2026-08-15</v>
       </c>
-      <c r="R5" t="str">
+      <c r="S5" t="str">
         <v/>
       </c>
     </row>
@@ -890,30 +905,33 @@
         <v>CA Phú Nhuận</v>
       </c>
       <c r="L6" t="str">
+        <v>56 Nguyễn Văn Trỗi, Phú Nhuận, TP.HCM</v>
+      </c>
+      <c r="M6" t="str">
         <v>2026-09-01</v>
       </c>
-      <c r="M6" t="str">
+      <c r="N6" t="str">
         <v>2027-08-31</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>5000000</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>2</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>10000000</v>
       </c>
-      <c r="Q6" t="str">
+      <c r="R6" t="str">
         <v>2026-09-01</v>
       </c>
-      <c r="R6" t="str">
+      <c r="S6" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
new excel file for import
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_tenant_draft_contracts.xlsx
+++ b/docs/SLMS2026_import_tenant_draft_contracts.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -564,16 +564,44 @@
         <v>101, 102, 103</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B21" t="str">
+        <v>MTX#11 NORENO full NT</v>
+      </c>
+      <c r="C21" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="D21" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>HD-MTX-13-RENO-RM-FULL</v>
+      </c>
+      <c r="B22" t="str">
+        <v>MTX#13 THEO_PHONG full NT</v>
+      </c>
+      <c r="C22" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="D22" t="str">
+        <v>101, 102, 103, 104</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D22"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -911,16 +939,128 @@
         <v>2026-09-01</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v>MTX#11 NORENO full NT</v>
+      </c>
+      <c r="D7" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>Vũ Gia Khang</v>
+      </c>
+      <c r="G7" t="str">
+        <v>079085001006</v>
+      </c>
+      <c r="H7" t="str">
+        <v>0901000006</v>
+      </c>
+      <c r="I7" t="str">
+        <v>1994-02-14</v>
+      </c>
+      <c r="J7" t="str">
+        <v>2018-09-10</v>
+      </c>
+      <c r="K7" t="str">
+        <v>CA Tân Bình</v>
+      </c>
+      <c r="L7" t="str">
+        <v>88 Cộng Hòa, Tân Bình, TP.HCM</v>
+      </c>
+      <c r="M7" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="N7" t="str">
+        <v>2027-09-30</v>
+      </c>
+      <c r="O7">
+        <v>11500000</v>
+      </c>
+      <c r="P7">
+        <v>2</v>
+      </c>
+      <c r="Q7">
+        <v>23000000</v>
+      </c>
+      <c r="R7" t="str">
+        <v>2026-10-01</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>HD-MTX-13-RENO-RM-FULL</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v>MTX#13 THEO_PHONG full NT</v>
+      </c>
+      <c r="D8" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E8" t="str">
+        <v>101</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Đỗ Minh Trang</v>
+      </c>
+      <c r="G8" t="str">
+        <v>079085001007</v>
+      </c>
+      <c r="H8" t="str">
+        <v>0901000007</v>
+      </c>
+      <c r="I8" t="str">
+        <v>1997-11-09</v>
+      </c>
+      <c r="J8" t="str">
+        <v>2021-04-22</v>
+      </c>
+      <c r="K8" t="str">
+        <v>CA Thủ Đức</v>
+      </c>
+      <c r="L8" t="str">
+        <v>120 Võ Văn Ngân, Thủ Đức, TP.HCM</v>
+      </c>
+      <c r="M8" t="str">
+        <v>2026-10-15</v>
+      </c>
+      <c r="N8" t="str">
+        <v>2027-10-14</v>
+      </c>
+      <c r="O8">
+        <v>5800000</v>
+      </c>
+      <c r="P8">
+        <v>1</v>
+      </c>
+      <c r="Q8">
+        <v>5800000</v>
+      </c>
+      <c r="R8" t="str">
+        <v>2026-10-15</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1020,9 +1160,37 @@
         <v>Phòng 101–103</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>HD-MTX-11-NORENO-FULL</v>
+      </c>
+      <c r="B8" t="str">
+        <v>MTX#11 NORENO full NT</v>
+      </c>
+      <c r="C8" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Case full nội thất, import đợt 1 là đủ</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>HD-MTX-13-RENO-RM-FULL</v>
+      </c>
+      <c r="B9" t="str">
+        <v>MTX#13 THEO_PHONG full NT</v>
+      </c>
+      <c r="C9" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Case full nội thất theo phòng 101–104</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix payos transfer pricing
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_tenant_draft_contracts.xlsx
+++ b/docs/SLMS2026_import_tenant_draft_contracts.xlsx
@@ -399,14 +399,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A21"/>
   <cols>
     <col min="1" max="1" width="110.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Hướng dẫn import HĐ thuê nháp (DRAFT) — 25 dòng map tenant01..25</v>
+        <v>Hướng dẫn import HĐ thuê nháp (DRAFT) — Demo nhận nhà 11/08/2026</v>
       </c>
     </row>
     <row r="2">
@@ -416,52 +416,102 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>1. Seed tài khoản: tenant01..tenant28 / 123456 (chưa thuê).</v>
+        <v>MỤC TIÊU DEMO (confirm OTP / kích hoạt HĐ ngày 11/08/2026)</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2. Import đợt 1: docs/SLMS2026_import_matrix_dot1.xlsx</v>
+        <v xml:space="preserve">  contract.max-early-move-in-days = 3 (application.yaml)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>3. Import đợt 2 (RENO): docs/SLMS2026_import_matrix_dot2.xlsx</v>
+        <v xml:space="preserve">  A (8 HĐ): Ngày vào ở = 2026-08-11 → onboard ĐÚNG NGÀY → OK</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>4. Import file này: POST /api/v1/import/tenant-draft-contracts-excel?dryRun=</v>
+        <v xml:space="preserve">  B (9 HĐ): Ngày vào ở = 12/13/14-08 → sớm 1–3 ngày → OK, BE ghi moveIn/start = 11/08, giữ endDate</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>5. Map BĐS: cột Mã HĐ inbound (= mã master) hoặc Tên tòa nhà.</v>
+        <v xml:space="preserve">  C (8 HĐ): Ngày vào ở ≥ 15/08 → sớm &gt;3 ngày → REJECT: "Chỉ được nhận nhà sớm tối đa 3 ngày..."</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>6. 15 NORENO nguyên căn + 5 RENO NGUYEN_CAN + 5 RENO THEO_PHONG phòng 101.</v>
+        <v xml:space="preserve">  Chi tiết case A1..C8: sheet 0. Tham_Chieu_BDS</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>7. SĐT/CCCD/họ tên khớp SampleDataSeeder tenant01..25.</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>8. tenant26..28 không có dòng nháp — dùng test gán tay.</v>
+        <v>QUY TRÌNH IMPORT</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>1. Seed tài khoản: tenant01..tenant28 / 123456 (chưa thuê).</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2. Import đợt 1: docs/SLMS2026_import_matrix_dot1.xlsx</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>3. Import đợt 2 (RENO): docs/SLMS2026_import_matrix_dot2.xlsx</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>4. Import file này: POST /api/v1/import/tenant-draft-contracts-excel?dryRun=</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>5. Map BĐS: cột Mã HĐ inbound (= mã master) hoặc Tên tòa nhà.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>6. 15 NORENO nguyên căn + 5 RENO NGUYEN_CAN + 5 RENO THEO_PHONG phòng 101.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>7. SĐT/CCCD/họ tên khớp SampleDataSeeder tenant01..25.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>8. tenant26..28 không có dòng nháp — dùng test gán tay.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
         <v>9. Nên dryRun=true trước; Auth ADMIN hoặc MANAGER.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>SCRIPT GỐC: node docs/generate-matrix-50.js (regenerate cả ma trận + draft)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -584,10 +634,10 @@
         <v>20 Lê Lợi, Quận 1</v>
       </c>
       <c r="M2" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
       <c r="N2" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-10</v>
       </c>
       <c r="O2">
         <v>14000000</v>
@@ -599,7 +649,7 @@
         <v>14000000</v>
       </c>
       <c r="R2" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
     </row>
     <row r="3">
@@ -640,10 +690,10 @@
         <v>21 Lê Lợi, Quận 3</v>
       </c>
       <c r="M3" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
       <c r="N3" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-10</v>
       </c>
       <c r="O3">
         <v>16000000</v>
@@ -655,7 +705,7 @@
         <v>32000000</v>
       </c>
       <c r="R3" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
     </row>
     <row r="4">
@@ -696,10 +746,10 @@
         <v>22 Lê Lợi, Bình Thạnh</v>
       </c>
       <c r="M4" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
       <c r="N4" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-10</v>
       </c>
       <c r="O4">
         <v>18000000</v>
@@ -711,7 +761,7 @@
         <v>18000000</v>
       </c>
       <c r="R4" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
     </row>
     <row r="5">
@@ -752,10 +802,10 @@
         <v>23 Lê Lợi, Gò Vấp</v>
       </c>
       <c r="M5" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
       <c r="N5" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-10</v>
       </c>
       <c r="O5">
         <v>20000000</v>
@@ -767,7 +817,7 @@
         <v>40000000</v>
       </c>
       <c r="R5" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
     </row>
     <row r="6">
@@ -808,10 +858,10 @@
         <v>24 Lê Lợi, Phú Nhuận</v>
       </c>
       <c r="M6" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
       <c r="N6" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-10</v>
       </c>
       <c r="O6">
         <v>22000000</v>
@@ -823,7 +873,7 @@
         <v>22000000</v>
       </c>
       <c r="R6" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
     </row>
     <row r="7">
@@ -864,10 +914,10 @@
         <v>25 Lê Lợi, Cầu Giấy</v>
       </c>
       <c r="M7" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
       <c r="N7" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-10</v>
       </c>
       <c r="O7">
         <v>24000000</v>
@@ -879,7 +929,7 @@
         <v>48000000</v>
       </c>
       <c r="R7" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
     </row>
     <row r="8">
@@ -920,10 +970,10 @@
         <v>26 Lê Lợi, Quận 1</v>
       </c>
       <c r="M8" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
       <c r="N8" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-10</v>
       </c>
       <c r="O8">
         <v>26000000</v>
@@ -935,7 +985,7 @@
         <v>26000000</v>
       </c>
       <c r="R8" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
     </row>
     <row r="9">
@@ -976,10 +1026,10 @@
         <v>27 Lê Lợi, Quận 3</v>
       </c>
       <c r="M9" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
       <c r="N9" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-10</v>
       </c>
       <c r="O9">
         <v>12000000</v>
@@ -991,7 +1041,7 @@
         <v>24000000</v>
       </c>
       <c r="R9" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-11</v>
       </c>
     </row>
     <row r="10">
@@ -1032,10 +1082,10 @@
         <v>28 Lê Lợi, Bình Thạnh</v>
       </c>
       <c r="M10" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-12</v>
       </c>
       <c r="N10" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-11</v>
       </c>
       <c r="O10">
         <v>14000000</v>
@@ -1047,7 +1097,7 @@
         <v>14000000</v>
       </c>
       <c r="R10" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="11">
@@ -1088,10 +1138,10 @@
         <v>29 Lê Lợi, Gò Vấp</v>
       </c>
       <c r="M11" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-12</v>
       </c>
       <c r="N11" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-11</v>
       </c>
       <c r="O11">
         <v>16000000</v>
@@ -1103,7 +1153,7 @@
         <v>32000000</v>
       </c>
       <c r="R11" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="12">
@@ -1144,10 +1194,10 @@
         <v>30 Lê Lợi, Phú Nhuận</v>
       </c>
       <c r="M12" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-12</v>
       </c>
       <c r="N12" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-11</v>
       </c>
       <c r="O12">
         <v>18000000</v>
@@ -1159,7 +1209,7 @@
         <v>18000000</v>
       </c>
       <c r="R12" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="13">
@@ -1200,10 +1250,10 @@
         <v>31 Lê Lợi, Cầu Giấy</v>
       </c>
       <c r="M13" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-13</v>
       </c>
       <c r="N13" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-12</v>
       </c>
       <c r="O13">
         <v>20000000</v>
@@ -1215,7 +1265,7 @@
         <v>40000000</v>
       </c>
       <c r="R13" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-13</v>
       </c>
     </row>
     <row r="14">
@@ -1256,10 +1306,10 @@
         <v>32 Lê Lợi, Quận 1</v>
       </c>
       <c r="M14" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-13</v>
       </c>
       <c r="N14" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-12</v>
       </c>
       <c r="O14">
         <v>22000000</v>
@@ -1271,7 +1321,7 @@
         <v>22000000</v>
       </c>
       <c r="R14" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-13</v>
       </c>
     </row>
     <row r="15">
@@ -1312,10 +1362,10 @@
         <v>33 Lê Lợi, Quận 3</v>
       </c>
       <c r="M15" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-13</v>
       </c>
       <c r="N15" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-12</v>
       </c>
       <c r="O15">
         <v>24000000</v>
@@ -1327,7 +1377,7 @@
         <v>48000000</v>
       </c>
       <c r="R15" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-13</v>
       </c>
     </row>
     <row r="16">
@@ -1368,10 +1418,10 @@
         <v>34 Lê Lợi, Bình Thạnh</v>
       </c>
       <c r="M16" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-14</v>
       </c>
       <c r="N16" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-13</v>
       </c>
       <c r="O16">
         <v>26000000</v>
@@ -1383,7 +1433,7 @@
         <v>26000000</v>
       </c>
       <c r="R16" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-14</v>
       </c>
     </row>
     <row r="17">
@@ -1424,10 +1474,10 @@
         <v>35 Lê Lợi, Gò Vấp</v>
       </c>
       <c r="M17" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-14</v>
       </c>
       <c r="N17" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-13</v>
       </c>
       <c r="O17">
         <v>12000000</v>
@@ -1439,7 +1489,7 @@
         <v>24000000</v>
       </c>
       <c r="R17" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-14</v>
       </c>
     </row>
     <row r="18">
@@ -1480,10 +1530,10 @@
         <v>36 Lê Lợi, Phú Nhuận</v>
       </c>
       <c r="M18" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-14</v>
       </c>
       <c r="N18" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-13</v>
       </c>
       <c r="O18">
         <v>14000000</v>
@@ -1495,7 +1545,7 @@
         <v>14000000</v>
       </c>
       <c r="R18" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-14</v>
       </c>
     </row>
     <row r="19">
@@ -1536,10 +1586,10 @@
         <v>37 Lê Lợi, Cầu Giấy</v>
       </c>
       <c r="M19" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-15</v>
       </c>
       <c r="N19" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-14</v>
       </c>
       <c r="O19">
         <v>16000000</v>
@@ -1551,7 +1601,7 @@
         <v>32000000</v>
       </c>
       <c r="R19" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-15</v>
       </c>
     </row>
     <row r="20">
@@ -1592,10 +1642,10 @@
         <v>38 Lê Lợi, Quận 1</v>
       </c>
       <c r="M20" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-15</v>
       </c>
       <c r="N20" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-14</v>
       </c>
       <c r="O20">
         <v>18000000</v>
@@ -1607,7 +1657,7 @@
         <v>18000000</v>
       </c>
       <c r="R20" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-15</v>
       </c>
     </row>
     <row r="21">
@@ -1648,10 +1698,10 @@
         <v>39 Lê Lợi, Quận 3</v>
       </c>
       <c r="M21" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-16</v>
       </c>
       <c r="N21" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-15</v>
       </c>
       <c r="O21">
         <v>20000000</v>
@@ -1663,7 +1713,7 @@
         <v>40000000</v>
       </c>
       <c r="R21" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-16</v>
       </c>
     </row>
     <row r="22">
@@ -1704,10 +1754,10 @@
         <v>40 Lê Lợi, Quận 3</v>
       </c>
       <c r="M22" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-16</v>
       </c>
       <c r="N22" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-15</v>
       </c>
       <c r="O22">
         <v>3300000</v>
@@ -1719,7 +1769,7 @@
         <v>3300000</v>
       </c>
       <c r="R22" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-16</v>
       </c>
     </row>
     <row r="23">
@@ -1760,10 +1810,10 @@
         <v>41 Lê Lợi, Bình Thạnh</v>
       </c>
       <c r="M23" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-18</v>
       </c>
       <c r="N23" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-17</v>
       </c>
       <c r="O23">
         <v>3700000</v>
@@ -1775,7 +1825,7 @@
         <v>7400000</v>
       </c>
       <c r="R23" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-18</v>
       </c>
     </row>
     <row r="24">
@@ -1816,10 +1866,10 @@
         <v>42 Lê Lợi, Gò Vấp</v>
       </c>
       <c r="M24" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-20</v>
       </c>
       <c r="N24" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-19</v>
       </c>
       <c r="O24">
         <v>4100000</v>
@@ -1831,7 +1881,7 @@
         <v>4100000</v>
       </c>
       <c r="R24" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-20</v>
       </c>
     </row>
     <row r="25">
@@ -1872,10 +1922,10 @@
         <v>43 Lê Lợi, Phú Nhuận</v>
       </c>
       <c r="M25" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-25</v>
       </c>
       <c r="N25" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-24</v>
       </c>
       <c r="O25">
         <v>4500000</v>
@@ -1887,7 +1937,7 @@
         <v>9000000</v>
       </c>
       <c r="R25" t="str">
-        <v>2026-10-01</v>
+        <v>2026-08-25</v>
       </c>
     </row>
     <row r="26">
@@ -1928,10 +1978,10 @@
         <v>44 Lê Lợi, Cầu Giấy</v>
       </c>
       <c r="M26" t="str">
-        <v>2026-10-01</v>
+        <v>2026-09-01</v>
       </c>
       <c r="N26" t="str">
-        <v>2027-09-30</v>
+        <v>2027-08-31</v>
       </c>
       <c r="O26">
         <v>2500000</v>
@@ -1943,7 +1993,7 @@
         <v>2500000</v>
       </c>
       <c r="R26" t="str">
-        <v>2026-10-01</v>
+        <v>2026-09-01</v>
       </c>
     </row>
   </sheetData>
@@ -1955,16 +2005,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:M26"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
-    <col min="2" max="2" width="36.83203125" customWidth="1"/>
-    <col min="3" max="3" width="32.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="36.83203125" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="36.83203125" customWidth="1"/>
+    <col min="13" max="13" width="36.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1972,25 +2027,40 @@
         <v>#</v>
       </c>
       <c r="B1" t="str">
+        <v>Case</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Nhóm demo</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Ngày vào ở (kế hoạch)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Ngày kết thúc</v>
+      </c>
+      <c r="F1" t="str">
         <v>Mã HĐ master</v>
       </c>
-      <c r="C1" t="str">
+      <c r="G1" t="str">
         <v>Tên tòa nhà</v>
       </c>
-      <c r="D1" t="str">
+      <c r="H1" t="str">
         <v>Loại</v>
       </c>
-      <c r="E1" t="str">
+      <c r="I1" t="str">
         <v>Số phòng</v>
       </c>
-      <c r="F1" t="str">
+      <c r="J1" t="str">
         <v>Tenant seed</v>
       </c>
-      <c r="G1" t="str">
+      <c r="K1" t="str">
         <v>SĐT</v>
       </c>
-      <c r="H1" t="str">
-        <v>Ghi chú</v>
+      <c r="L1" t="str">
+        <v>Kỳ vọng confirm 11/08</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Ghi chú BĐS</v>
       </c>
     </row>
     <row r="2">
@@ -1998,24 +2068,39 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
+        <v>A1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ĐÚNG NGÀY</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F2" t="str">
         <v>HD-MTX-01-NORENO-WH-NONE</v>
       </c>
-      <c r="C2" t="str">
+      <c r="G2" t="str">
         <v>MTX#01 NGUYEN_CAN NONE</v>
       </c>
-      <c r="D2" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E2" t="str">
+      <c r="H2" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I2" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F2" t="str">
+      <c r="J2" t="str">
         <v>tenant01</v>
       </c>
-      <c r="G2" t="str">
+      <c r="K2" t="str">
         <v>0904000001</v>
       </c>
-      <c r="H2" t="str">
+      <c r="L2" t="str">
+        <v>OK confirm 11/08</v>
+      </c>
+      <c r="M2" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2024,24 +2109,39 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
+        <v>A2</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ĐÚNG NGÀY</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F3" t="str">
         <v>HD-MTX-02-NORENO-WH-NONE</v>
       </c>
-      <c r="C3" t="str">
+      <c r="G3" t="str">
         <v>MTX#02 NGUYEN_CAN NONE</v>
       </c>
-      <c r="D3" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E3" t="str">
+      <c r="H3" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I3" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F3" t="str">
+      <c r="J3" t="str">
         <v>tenant02</v>
       </c>
-      <c r="G3" t="str">
+      <c r="K3" t="str">
         <v>0904000002</v>
       </c>
-      <c r="H3" t="str">
+      <c r="L3" t="str">
+        <v>OK confirm 11/08</v>
+      </c>
+      <c r="M3" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2050,24 +2150,39 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
+        <v>A3</v>
+      </c>
+      <c r="C4" t="str">
+        <v>ĐÚNG NGÀY</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F4" t="str">
         <v>HD-MTX-03-NORENO-WH-NONE</v>
       </c>
-      <c r="C4" t="str">
+      <c r="G4" t="str">
         <v>MTX#03 NGUYEN_CAN NONE</v>
       </c>
-      <c r="D4" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E4" t="str">
+      <c r="H4" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I4" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F4" t="str">
+      <c r="J4" t="str">
         <v>tenant03</v>
       </c>
-      <c r="G4" t="str">
+      <c r="K4" t="str">
         <v>0904000003</v>
       </c>
-      <c r="H4" t="str">
+      <c r="L4" t="str">
+        <v>OK confirm 11/08</v>
+      </c>
+      <c r="M4" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2076,24 +2191,39 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
+        <v>A4</v>
+      </c>
+      <c r="C5" t="str">
+        <v>ĐÚNG NGÀY</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F5" t="str">
         <v>HD-MTX-04-NORENO-WH-NONE</v>
       </c>
-      <c r="C5" t="str">
+      <c r="G5" t="str">
         <v>MTX#04 NGUYEN_CAN NONE</v>
       </c>
-      <c r="D5" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E5" t="str">
+      <c r="H5" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I5" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F5" t="str">
+      <c r="J5" t="str">
         <v>tenant04</v>
       </c>
-      <c r="G5" t="str">
+      <c r="K5" t="str">
         <v>0904000004</v>
       </c>
-      <c r="H5" t="str">
+      <c r="L5" t="str">
+        <v>OK confirm 11/08</v>
+      </c>
+      <c r="M5" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2102,24 +2232,39 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
+        <v>A5</v>
+      </c>
+      <c r="C6" t="str">
+        <v>ĐÚNG NGÀY</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F6" t="str">
         <v>HD-MTX-05-NORENO-WH-NONE</v>
       </c>
-      <c r="C6" t="str">
+      <c r="G6" t="str">
         <v>MTX#05 NGUYEN_CAN NONE</v>
       </c>
-      <c r="D6" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E6" t="str">
+      <c r="H6" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I6" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F6" t="str">
+      <c r="J6" t="str">
         <v>tenant05</v>
       </c>
-      <c r="G6" t="str">
+      <c r="K6" t="str">
         <v>0904000005</v>
       </c>
-      <c r="H6" t="str">
+      <c r="L6" t="str">
+        <v>OK confirm 11/08</v>
+      </c>
+      <c r="M6" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2128,24 +2273,39 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
+        <v>A6</v>
+      </c>
+      <c r="C7" t="str">
+        <v>ĐÚNG NGÀY</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F7" t="str">
         <v>HD-MTX-06-NORENO-WH-BASIC</v>
       </c>
-      <c r="C7" t="str">
+      <c r="G7" t="str">
         <v>MTX#06 NGUYEN_CAN BASIC</v>
       </c>
-      <c r="D7" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E7" t="str">
+      <c r="H7" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I7" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F7" t="str">
+      <c r="J7" t="str">
         <v>tenant06</v>
       </c>
-      <c r="G7" t="str">
+      <c r="K7" t="str">
         <v>0904000006</v>
       </c>
-      <c r="H7" t="str">
+      <c r="L7" t="str">
+        <v>OK confirm 11/08</v>
+      </c>
+      <c r="M7" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2154,24 +2314,39 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
+        <v>A7</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ĐÚNG NGÀY</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F8" t="str">
         <v>HD-MTX-07-NORENO-WH-BASIC</v>
       </c>
-      <c r="C8" t="str">
+      <c r="G8" t="str">
         <v>MTX#07 NGUYEN_CAN BASIC</v>
       </c>
-      <c r="D8" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E8" t="str">
+      <c r="H8" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I8" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F8" t="str">
+      <c r="J8" t="str">
         <v>tenant07</v>
       </c>
-      <c r="G8" t="str">
+      <c r="K8" t="str">
         <v>0904000007</v>
       </c>
-      <c r="H8" t="str">
+      <c r="L8" t="str">
+        <v>OK confirm 11/08</v>
+      </c>
+      <c r="M8" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2180,24 +2355,39 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
+        <v>A8</v>
+      </c>
+      <c r="C9" t="str">
+        <v>ĐÚNG NGÀY</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F9" t="str">
         <v>HD-MTX-08-NORENO-WH-BASIC</v>
       </c>
-      <c r="C9" t="str">
+      <c r="G9" t="str">
         <v>MTX#08 NGUYEN_CAN BASIC</v>
       </c>
-      <c r="D9" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E9" t="str">
+      <c r="H9" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I9" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F9" t="str">
+      <c r="J9" t="str">
         <v>tenant08</v>
       </c>
-      <c r="G9" t="str">
+      <c r="K9" t="str">
         <v>0904000008</v>
       </c>
-      <c r="H9" t="str">
+      <c r="L9" t="str">
+        <v>OK confirm 11/08</v>
+      </c>
+      <c r="M9" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2206,24 +2396,39 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C10" t="str">
+        <v>SỚM ≤3N (+1)</v>
+      </c>
+      <c r="D10" t="str">
+        <v>2026-08-12</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2027-08-11</v>
+      </c>
+      <c r="F10" t="str">
         <v>HD-MTX-09-NORENO-WH-BASIC</v>
       </c>
-      <c r="C10" t="str">
+      <c r="G10" t="str">
         <v>MTX#09 NGUYEN_CAN BASIC</v>
       </c>
-      <c r="D10" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E10" t="str">
+      <c r="H10" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I10" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F10" t="str">
+      <c r="J10" t="str">
         <v>tenant09</v>
       </c>
-      <c r="G10" t="str">
+      <c r="K10" t="str">
         <v>0904000009</v>
       </c>
-      <c r="H10" t="str">
+      <c r="L10" t="str">
+        <v>OK sớm 1 ngày → moveIn=11/08</v>
+      </c>
+      <c r="M10" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2232,24 +2437,39 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
+        <v>B2</v>
+      </c>
+      <c r="C11" t="str">
+        <v>SỚM ≤3N (+1)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>2026-08-12</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2027-08-11</v>
+      </c>
+      <c r="F11" t="str">
         <v>HD-MTX-10-NORENO-WH-BASIC</v>
       </c>
-      <c r="C11" t="str">
+      <c r="G11" t="str">
         <v>MTX#10 NGUYEN_CAN BASIC</v>
       </c>
-      <c r="D11" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E11" t="str">
+      <c r="H11" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I11" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F11" t="str">
+      <c r="J11" t="str">
         <v>tenant10</v>
       </c>
-      <c r="G11" t="str">
+      <c r="K11" t="str">
         <v>0904000010</v>
       </c>
-      <c r="H11" t="str">
+      <c r="L11" t="str">
+        <v>OK sớm 1 ngày → moveIn=11/08</v>
+      </c>
+      <c r="M11" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2258,24 +2478,39 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
+        <v>B3</v>
+      </c>
+      <c r="C12" t="str">
+        <v>SỚM ≤3N (+1)</v>
+      </c>
+      <c r="D12" t="str">
+        <v>2026-08-12</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2027-08-11</v>
+      </c>
+      <c r="F12" t="str">
         <v>HD-MTX-11-NORENO-WH-FULL</v>
       </c>
-      <c r="C12" t="str">
+      <c r="G12" t="str">
         <v>MTX#11 NGUYEN_CAN FULL</v>
       </c>
-      <c r="D12" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E12" t="str">
+      <c r="H12" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I12" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F12" t="str">
+      <c r="J12" t="str">
         <v>tenant11</v>
       </c>
-      <c r="G12" t="str">
+      <c r="K12" t="str">
         <v>0904000011</v>
       </c>
-      <c r="H12" t="str">
+      <c r="L12" t="str">
+        <v>OK sớm 1 ngày → moveIn=11/08</v>
+      </c>
+      <c r="M12" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2284,24 +2519,39 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
+        <v>B4</v>
+      </c>
+      <c r="C13" t="str">
+        <v>SỚM ≤3N (+2)</v>
+      </c>
+      <c r="D13" t="str">
+        <v>2026-08-13</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2027-08-12</v>
+      </c>
+      <c r="F13" t="str">
         <v>HD-MTX-12-NORENO-WH-FULL</v>
       </c>
-      <c r="C13" t="str">
+      <c r="G13" t="str">
         <v>MTX#12 NGUYEN_CAN FULL</v>
       </c>
-      <c r="D13" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E13" t="str">
+      <c r="H13" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I13" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F13" t="str">
+      <c r="J13" t="str">
         <v>tenant12</v>
       </c>
-      <c r="G13" t="str">
+      <c r="K13" t="str">
         <v>0904000012</v>
       </c>
-      <c r="H13" t="str">
+      <c r="L13" t="str">
+        <v>OK sớm 2 ngày → moveIn=11/08</v>
+      </c>
+      <c r="M13" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2310,24 +2560,39 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
+        <v>B5</v>
+      </c>
+      <c r="C14" t="str">
+        <v>SỚM ≤3N (+2)</v>
+      </c>
+      <c r="D14" t="str">
+        <v>2026-08-13</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2027-08-12</v>
+      </c>
+      <c r="F14" t="str">
         <v>HD-MTX-13-NORENO-WH-FULL</v>
       </c>
-      <c r="C14" t="str">
+      <c r="G14" t="str">
         <v>MTX#13 NGUYEN_CAN FULL</v>
       </c>
-      <c r="D14" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E14" t="str">
+      <c r="H14" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I14" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F14" t="str">
+      <c r="J14" t="str">
         <v>tenant13</v>
       </c>
-      <c r="G14" t="str">
+      <c r="K14" t="str">
         <v>0904000013</v>
       </c>
-      <c r="H14" t="str">
+      <c r="L14" t="str">
+        <v>OK sớm 2 ngày → moveIn=11/08</v>
+      </c>
+      <c r="M14" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2336,24 +2601,39 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
+        <v>B6</v>
+      </c>
+      <c r="C15" t="str">
+        <v>SỚM ≤3N (+2)</v>
+      </c>
+      <c r="D15" t="str">
+        <v>2026-08-13</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2027-08-12</v>
+      </c>
+      <c r="F15" t="str">
         <v>HD-MTX-14-NORENO-WH-FULL</v>
       </c>
-      <c r="C15" t="str">
+      <c r="G15" t="str">
         <v>MTX#14 NGUYEN_CAN FULL</v>
       </c>
-      <c r="D15" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E15" t="str">
+      <c r="H15" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I15" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F15" t="str">
+      <c r="J15" t="str">
         <v>tenant14</v>
       </c>
-      <c r="G15" t="str">
+      <c r="K15" t="str">
         <v>0904000014</v>
       </c>
-      <c r="H15" t="str">
+      <c r="L15" t="str">
+        <v>OK sớm 2 ngày → moveIn=11/08</v>
+      </c>
+      <c r="M15" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2362,24 +2642,39 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
+        <v>B7</v>
+      </c>
+      <c r="C16" t="str">
+        <v>SỚM ≤3N (+3)</v>
+      </c>
+      <c r="D16" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2027-08-13</v>
+      </c>
+      <c r="F16" t="str">
         <v>HD-MTX-15-NORENO-WH-FULL</v>
       </c>
-      <c r="C16" t="str">
+      <c r="G16" t="str">
         <v>MTX#15 NGUYEN_CAN FULL</v>
       </c>
-      <c r="D16" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E16" t="str">
+      <c r="H16" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I16" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F16" t="str">
+      <c r="J16" t="str">
         <v>tenant15</v>
       </c>
-      <c r="G16" t="str">
+      <c r="K16" t="str">
         <v>0904000015</v>
       </c>
-      <c r="H16" t="str">
+      <c r="L16" t="str">
+        <v>OK sớm 3 ngày (biên) → moveIn=11/08</v>
+      </c>
+      <c r="M16" t="str">
         <v>Sẵn sau đợt 1 (NORENO)</v>
       </c>
     </row>
@@ -2388,24 +2683,39 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
+        <v>B8</v>
+      </c>
+      <c r="C17" t="str">
+        <v>SỚM ≤3N (+3)</v>
+      </c>
+      <c r="D17" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="E17" t="str">
+        <v>2027-08-13</v>
+      </c>
+      <c r="F17" t="str">
         <v>HD-MTX-16-RENO-WH-NONE</v>
       </c>
-      <c r="C17" t="str">
+      <c r="G17" t="str">
         <v>MTX#16 NGUYEN_CAN NONE</v>
       </c>
-      <c r="D17" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E17" t="str">
+      <c r="H17" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I17" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F17" t="str">
+      <c r="J17" t="str">
         <v>tenant16</v>
       </c>
-      <c r="G17" t="str">
+      <c r="K17" t="str">
         <v>0904000016</v>
       </c>
-      <c r="H17" t="str">
+      <c r="L17" t="str">
+        <v>OK sớm 3 ngày (biên) → moveIn=11/08</v>
+      </c>
+      <c r="M17" t="str">
         <v>Cần import đợt 2 (NGUYEN_CAN) trước</v>
       </c>
     </row>
@@ -2414,24 +2724,39 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
+        <v>B9</v>
+      </c>
+      <c r="C18" t="str">
+        <v>SỚM ≤3N (+3)</v>
+      </c>
+      <c r="D18" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="E18" t="str">
+        <v>2027-08-13</v>
+      </c>
+      <c r="F18" t="str">
         <v>HD-MTX-17-RENO-WH-NONE</v>
       </c>
-      <c r="C18" t="str">
+      <c r="G18" t="str">
         <v>MTX#17 NGUYEN_CAN NONE</v>
       </c>
-      <c r="D18" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E18" t="str">
+      <c r="H18" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I18" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F18" t="str">
+      <c r="J18" t="str">
         <v>tenant17</v>
       </c>
-      <c r="G18" t="str">
+      <c r="K18" t="str">
         <v>0904000017</v>
       </c>
-      <c r="H18" t="str">
+      <c r="L18" t="str">
+        <v>OK sớm 3 ngày (biên) → moveIn=11/08</v>
+      </c>
+      <c r="M18" t="str">
         <v>Cần import đợt 2 (NGUYEN_CAN) trước</v>
       </c>
     </row>
@@ -2440,24 +2765,39 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
+        <v>C1</v>
+      </c>
+      <c r="C19" t="str">
+        <v>SỚM &gt;3N (+4)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>2026-08-15</v>
+      </c>
+      <c r="E19" t="str">
+        <v>2027-08-14</v>
+      </c>
+      <c r="F19" t="str">
         <v>HD-MTX-18-RENO-WH-NONE</v>
       </c>
-      <c r="C19" t="str">
+      <c r="G19" t="str">
         <v>MTX#18 NGUYEN_CAN NONE</v>
       </c>
-      <c r="D19" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E19" t="str">
+      <c r="H19" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I19" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F19" t="str">
+      <c r="J19" t="str">
         <v>tenant18</v>
       </c>
-      <c r="G19" t="str">
+      <c r="K19" t="str">
         <v>0904000018</v>
       </c>
-      <c r="H19" t="str">
+      <c r="L19" t="str">
+        <v>REJECT confirm 11/08 (sớm 4 ngày)</v>
+      </c>
+      <c r="M19" t="str">
         <v>Cần import đợt 2 (NGUYEN_CAN) trước</v>
       </c>
     </row>
@@ -2466,24 +2806,39 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
+        <v>C2</v>
+      </c>
+      <c r="C20" t="str">
+        <v>SỚM &gt;3N (+4)</v>
+      </c>
+      <c r="D20" t="str">
+        <v>2026-08-15</v>
+      </c>
+      <c r="E20" t="str">
+        <v>2027-08-14</v>
+      </c>
+      <c r="F20" t="str">
         <v>HD-MTX-19-RENO-WH-BASIC-HO</v>
       </c>
-      <c r="C20" t="str">
+      <c r="G20" t="str">
         <v>MTX#19 NGUYEN_CAN BASIC</v>
       </c>
-      <c r="D20" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E20" t="str">
+      <c r="H20" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I20" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F20" t="str">
+      <c r="J20" t="str">
         <v>tenant19</v>
       </c>
-      <c r="G20" t="str">
+      <c r="K20" t="str">
         <v>0904000019</v>
       </c>
-      <c r="H20" t="str">
+      <c r="L20" t="str">
+        <v>REJECT confirm 11/08 (sớm 4 ngày)</v>
+      </c>
+      <c r="M20" t="str">
         <v>Cần import đợt 2 (NGUYEN_CAN) trước</v>
       </c>
     </row>
@@ -2492,24 +2847,39 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
+        <v>C3</v>
+      </c>
+      <c r="C21" t="str">
+        <v>SỚM &gt;3N (+5)</v>
+      </c>
+      <c r="D21" t="str">
+        <v>2026-08-16</v>
+      </c>
+      <c r="E21" t="str">
+        <v>2027-08-15</v>
+      </c>
+      <c r="F21" t="str">
         <v>HD-MTX-20-RENO-WH-BASIC-HO</v>
       </c>
-      <c r="C21" t="str">
+      <c r="G21" t="str">
         <v>MTX#20 NGUYEN_CAN BASIC</v>
       </c>
-      <c r="D21" t="str">
-        <v>NGUYEN_CAN</v>
-      </c>
-      <c r="E21" t="str">
+      <c r="H21" t="str">
+        <v>NGUYEN_CAN</v>
+      </c>
+      <c r="I21" t="str">
         <v>(nguyên căn)</v>
       </c>
-      <c r="F21" t="str">
+      <c r="J21" t="str">
         <v>tenant20</v>
       </c>
-      <c r="G21" t="str">
+      <c r="K21" t="str">
         <v>0904000020</v>
       </c>
-      <c r="H21" t="str">
+      <c r="L21" t="str">
+        <v>REJECT confirm 11/08 (sớm 5 ngày)</v>
+      </c>
+      <c r="M21" t="str">
         <v>Cần import đợt 2 (NGUYEN_CAN) trước</v>
       </c>
     </row>
@@ -2518,24 +2888,39 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
+        <v>C4</v>
+      </c>
+      <c r="C22" t="str">
+        <v>SỚM &gt;3N (+5)</v>
+      </c>
+      <c r="D22" t="str">
+        <v>2026-08-16</v>
+      </c>
+      <c r="E22" t="str">
+        <v>2027-08-15</v>
+      </c>
+      <c r="F22" t="str">
         <v>HD-MTX-32-RENO-RM-NONE</v>
       </c>
-      <c r="C22" t="str">
+      <c r="G22" t="str">
         <v>MTX#32 THEO_PHONG NONE</v>
       </c>
-      <c r="D22" t="str">
+      <c r="H22" t="str">
         <v>THEO_PHONG</v>
       </c>
-      <c r="E22" t="str">
+      <c r="I22" t="str">
         <v>101</v>
       </c>
-      <c r="F22" t="str">
+      <c r="J22" t="str">
         <v>tenant21</v>
       </c>
-      <c r="G22" t="str">
+      <c r="K22" t="str">
         <v>0904000021</v>
       </c>
-      <c r="H22" t="str">
+      <c r="L22" t="str">
+        <v>REJECT confirm 11/08 (sớm 5 ngày)</v>
+      </c>
+      <c r="M22" t="str">
         <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101</v>
       </c>
     </row>
@@ -2544,24 +2929,39 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
+        <v>C5</v>
+      </c>
+      <c r="C23" t="str">
+        <v>SỚM &gt;3N (+7)</v>
+      </c>
+      <c r="D23" t="str">
+        <v>2026-08-18</v>
+      </c>
+      <c r="E23" t="str">
+        <v>2027-08-17</v>
+      </c>
+      <c r="F23" t="str">
         <v>HD-MTX-33-RENO-RM-NONE</v>
       </c>
-      <c r="C23" t="str">
+      <c r="G23" t="str">
         <v>MTX#33 THEO_PHONG NONE</v>
       </c>
-      <c r="D23" t="str">
+      <c r="H23" t="str">
         <v>THEO_PHONG</v>
       </c>
-      <c r="E23" t="str">
+      <c r="I23" t="str">
         <v>101</v>
       </c>
-      <c r="F23" t="str">
+      <c r="J23" t="str">
         <v>tenant22</v>
       </c>
-      <c r="G23" t="str">
+      <c r="K23" t="str">
         <v>0904000022</v>
       </c>
-      <c r="H23" t="str">
+      <c r="L23" t="str">
+        <v>REJECT confirm 11/08 (sớm 7 ngày)</v>
+      </c>
+      <c r="M23" t="str">
         <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101</v>
       </c>
     </row>
@@ -2570,24 +2970,39 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
+        <v>C6</v>
+      </c>
+      <c r="C24" t="str">
+        <v>SỚM &gt;3N (+9)</v>
+      </c>
+      <c r="D24" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="E24" t="str">
+        <v>2027-08-19</v>
+      </c>
+      <c r="F24" t="str">
         <v>HD-MTX-34-RENO-RM-NONE</v>
       </c>
-      <c r="C24" t="str">
+      <c r="G24" t="str">
         <v>MTX#34 THEO_PHONG NONE</v>
       </c>
-      <c r="D24" t="str">
+      <c r="H24" t="str">
         <v>THEO_PHONG</v>
       </c>
-      <c r="E24" t="str">
+      <c r="I24" t="str">
         <v>101</v>
       </c>
-      <c r="F24" t="str">
+      <c r="J24" t="str">
         <v>tenant23</v>
       </c>
-      <c r="G24" t="str">
+      <c r="K24" t="str">
         <v>0904000023</v>
       </c>
-      <c r="H24" t="str">
+      <c r="L24" t="str">
+        <v>REJECT confirm 11/08 (sớm 9 ngày)</v>
+      </c>
+      <c r="M24" t="str">
         <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101</v>
       </c>
     </row>
@@ -2596,24 +3011,39 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
+        <v>C7</v>
+      </c>
+      <c r="C25" t="str">
+        <v>SỚM &gt;3N (+14)</v>
+      </c>
+      <c r="D25" t="str">
+        <v>2026-08-25</v>
+      </c>
+      <c r="E25" t="str">
+        <v>2027-08-24</v>
+      </c>
+      <c r="F25" t="str">
         <v>HD-MTX-35-RENO-RM-NONE</v>
       </c>
-      <c r="C25" t="str">
+      <c r="G25" t="str">
         <v>MTX#35 THEO_PHONG NONE</v>
       </c>
-      <c r="D25" t="str">
+      <c r="H25" t="str">
         <v>THEO_PHONG</v>
       </c>
-      <c r="E25" t="str">
+      <c r="I25" t="str">
         <v>101</v>
       </c>
-      <c r="F25" t="str">
+      <c r="J25" t="str">
         <v>tenant24</v>
       </c>
-      <c r="G25" t="str">
+      <c r="K25" t="str">
         <v>0904000024</v>
       </c>
-      <c r="H25" t="str">
+      <c r="L25" t="str">
+        <v>REJECT confirm 11/08 (sớm 14 ngày)</v>
+      </c>
+      <c r="M25" t="str">
         <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101</v>
       </c>
     </row>
@@ -2622,30 +3052,45 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
+        <v>C8</v>
+      </c>
+      <c r="C26" t="str">
+        <v>SỚM &gt;3N (+21)</v>
+      </c>
+      <c r="D26" t="str">
+        <v>2026-09-01</v>
+      </c>
+      <c r="E26" t="str">
+        <v>2027-08-31</v>
+      </c>
+      <c r="F26" t="str">
         <v>HD-MTX-36-RENO-RM-BASIC-HO</v>
       </c>
-      <c r="C26" t="str">
+      <c r="G26" t="str">
         <v>MTX#36 THEO_PHONG BASIC</v>
       </c>
-      <c r="D26" t="str">
+      <c r="H26" t="str">
         <v>THEO_PHONG</v>
       </c>
-      <c r="E26" t="str">
+      <c r="I26" t="str">
         <v>101</v>
       </c>
-      <c r="F26" t="str">
+      <c r="J26" t="str">
         <v>tenant25</v>
       </c>
-      <c r="G26" t="str">
+      <c r="K26" t="str">
         <v>0904000025</v>
       </c>
-      <c r="H26" t="str">
+      <c r="L26" t="str">
+        <v>REJECT confirm 11/08 (sớm ~3 tuần)</v>
+      </c>
+      <c r="M26" t="str">
         <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
new excel import file v2
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_tenant_draft_contracts.xlsx
+++ b/docs/SLMS2026_import_tenant_draft_contracts.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A26"/>
   <cols>
     <col min="1" max="1" width="110.83203125" customWidth="1"/>
   </cols>
@@ -416,109 +416,134 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>MỤC TIÊU DEMO (confirm OTP / kích hoạt HĐ ngày 11/08/2026)</v>
+        <v>PHẠM VI: 36 HĐ nháp = 25 gốc + 11 HĐ thêm MTX#40..#50.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v xml:space="preserve">  contract.max-early-move-in-days = 3 (application.yaml)</v>
+        <v xml:space="preserve">  1–15: NORENO nguyên căn (sẵn sau đợt 1)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v xml:space="preserve">  A (8 HĐ): Ngày vào ở = 2026-08-11 → onboard ĐÚNG NGÀY → OK</v>
+        <v xml:space="preserve">  16–20: RENO NGUYEN_CAN (cần đợt 2)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v xml:space="preserve">  B (9 HĐ): Ngày vào ở = 12/13/14-08 → sớm 1–3 ngày → OK, BE ghi moveIn/start = 11/08, giữ endDate</v>
+        <v xml:space="preserve">  21–25: RENO THEO_PHONG phòng 101 — MTX#32..#36 (cần đợt 2)</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v xml:space="preserve">  C (8 HĐ): Ngày vào ở ≥ 15/08 → sớm &gt;3 ngày → REJECT: "Chỉ được nhận nhà sớm tối đa 3 ngày..."</v>
+        <v xml:space="preserve">  26–36: RENO THEO_PHONG phòng 101 — MTX#40..#50 (cần đợt 2)</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v xml:space="preserve">  Chi tiết case A1..C8: sheet 0. Tham_Chieu_BDS</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v/>
+        <v>MỤC TIÊU DEMO (confirm OTP / kích hoạt HĐ ngày 11/08/2026)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>QUY TRÌNH IMPORT</v>
+        <v xml:space="preserve">  contract.max-early-move-in-days = 3 (application.yaml)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>1. Seed tài khoản: tenant01..tenant28 / 123456 (chưa thuê).</v>
+        <v xml:space="preserve">  A (8 HĐ): Ngày vào ở = 2026-08-11 → OK đúng ngày</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2. Import đợt 1: docs/SLMS2026_import_matrix_dot1.xlsx</v>
+        <v xml:space="preserve">  B (9 HĐ): Ngày vào ở = 12/13/14-08 → sớm 1–3 ngày → OK</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>3. Import đợt 2 (RENO): docs/SLMS2026_import_matrix_dot2.xlsx</v>
+        <v xml:space="preserve">  C (8 HĐ): Ngày vào ở ≥ 15/08 → sớm &gt;3 ngày → REJECT</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>4. Import file này: POST /api/v1/import/tenant-draft-contracts-excel?dryRun=</v>
+        <v xml:space="preserve">  D (11 HĐ MTX#40..#50): Ngày vào ở = 2026-08-11 → OK đúng ngày</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>5. Map BĐS: cột Mã HĐ inbound (= mã master) hoặc Tên tòa nhà.</v>
+        <v xml:space="preserve">  Chi tiết: sheet 0. Tham_Chieu_BDS</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>6. 15 NORENO nguyên căn + 5 RENO NGUYEN_CAN + 5 RENO THEO_PHONG phòng 101.</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>7. SĐT/CCCD/họ tên khớp SampleDataSeeder tenant01..25.</v>
+        <v>QUY TRÌNH IMPORT</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>8. tenant26..28 không có dòng nháp — dùng test gán tay.</v>
+        <v>1. Seed tài khoản: tenant01..tenant36 / 123456 (SampleDataSeeder TENANT_COUNT).</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>9. Nên dryRun=true trước; Auth ADMIN hoặc MANAGER.</v>
+        <v>2. Import đợt 1: docs/SLMS2026_import_matrix_dot1.xlsx</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v/>
+        <v>3. Import đợt 2 (RENO): docs/SLMS2026_import_matrix_dot2.xlsx</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SCRIPT GỐC: node docs/generate-matrix-50.js (regenerate cả ma trận + draft)</v>
+        <v>4. Import file này: POST /api/v1/import/tenant-draft-contracts-excel?dryRun=</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>5. Map BĐS: cột Mã HĐ inbound (= mã master) hoặc Tên tòa nhà.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>6. SĐT/CCCD/họ tên khớp SampleDataSeeder tenant01..36.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>7. Nên dryRun=true trước; Auth ADMIN hoặc MANAGER.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>SCRIPT GỐC: node docs/generate-matrix-50.js</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A26"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:R37"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1996,16 +2021,632 @@
         <v>2026-09-01</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>HD-MTX-40-RENO-RM-BASIC-BUY</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v>MTX#40 THEO_PHONG BASIC</v>
+      </c>
+      <c r="D27" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E27" t="str">
+        <v>101</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Vũ Thị Giang</v>
+      </c>
+      <c r="G27" t="str">
+        <v>079000000026</v>
+      </c>
+      <c r="H27" t="str">
+        <v>0904000026</v>
+      </c>
+      <c r="I27" t="str">
+        <v>1989-02-10</v>
+      </c>
+      <c r="J27" t="str">
+        <v>2019-02-20</v>
+      </c>
+      <c r="K27" t="str">
+        <v>CA TP. Hồ Chí Minh</v>
+      </c>
+      <c r="L27" t="str">
+        <v>45 Lê Lợi, Gò Vấp</v>
+      </c>
+      <c r="M27" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="N27" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="O27">
+        <v>4100000</v>
+      </c>
+      <c r="P27">
+        <v>2</v>
+      </c>
+      <c r="Q27">
+        <v>8200000</v>
+      </c>
+      <c r="R27" t="str">
+        <v>2026-08-11</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>HD-MTX-41-RENO-RM-BASIC-BUY</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v>MTX#41 THEO_PHONG BASIC</v>
+      </c>
+      <c r="D28" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E28" t="str">
+        <v>101</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Đặng Thị Hà</v>
+      </c>
+      <c r="G28" t="str">
+        <v>079000000027</v>
+      </c>
+      <c r="H28" t="str">
+        <v>0904000027</v>
+      </c>
+      <c r="I28" t="str">
+        <v>1990-03-11</v>
+      </c>
+      <c r="J28" t="str">
+        <v>2020-03-21</v>
+      </c>
+      <c r="K28" t="str">
+        <v>CA Quận 1</v>
+      </c>
+      <c r="L28" t="str">
+        <v>46 Lê Lợi, Phú Nhuận</v>
+      </c>
+      <c r="M28" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="N28" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="O28">
+        <v>4500000</v>
+      </c>
+      <c r="P28">
+        <v>1</v>
+      </c>
+      <c r="Q28">
+        <v>4500000</v>
+      </c>
+      <c r="R28" t="str">
+        <v>2026-08-11</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>HD-MTX-42-RENO-RM-BASIC-BUY</v>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v>MTX#42 THEO_PHONG BASIC</v>
+      </c>
+      <c r="D29" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E29" t="str">
+        <v>101</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Bùi Thị Hiếu</v>
+      </c>
+      <c r="G29" t="str">
+        <v>079000000028</v>
+      </c>
+      <c r="H29" t="str">
+        <v>0904000028</v>
+      </c>
+      <c r="I29" t="str">
+        <v>1991-04-12</v>
+      </c>
+      <c r="J29" t="str">
+        <v>2021-04-22</v>
+      </c>
+      <c r="K29" t="str">
+        <v>CA Bình Thạnh</v>
+      </c>
+      <c r="L29" t="str">
+        <v>47 Lê Lợi, Cầu Giấy</v>
+      </c>
+      <c r="M29" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="N29" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="O29">
+        <v>2500000</v>
+      </c>
+      <c r="P29">
+        <v>2</v>
+      </c>
+      <c r="Q29">
+        <v>5000000</v>
+      </c>
+      <c r="R29" t="str">
+        <v>2026-08-11</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>HD-MTX-43-RENO-RM-BASIC-BUY</v>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v>MTX#43 THEO_PHONG BASIC</v>
+      </c>
+      <c r="D30" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E30" t="str">
+        <v>101</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Đỗ Thị Khoa</v>
+      </c>
+      <c r="G30" t="str">
+        <v>079000000029</v>
+      </c>
+      <c r="H30" t="str">
+        <v>0904000029</v>
+      </c>
+      <c r="I30" t="str">
+        <v>1992-05-13</v>
+      </c>
+      <c r="J30" t="str">
+        <v>2022-05-23</v>
+      </c>
+      <c r="K30" t="str">
+        <v>CA Gò Vấp</v>
+      </c>
+      <c r="L30" t="str">
+        <v>48 Lê Lợi, Quận 1</v>
+      </c>
+      <c r="M30" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="N30" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="O30">
+        <v>2900000</v>
+      </c>
+      <c r="P30">
+        <v>1</v>
+      </c>
+      <c r="Q30">
+        <v>2900000</v>
+      </c>
+      <c r="R30" t="str">
+        <v>2026-08-11</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>HD-MTX-44-RENO-RM-FULL</v>
+      </c>
+      <c r="B31" t="str">
+        <v/>
+      </c>
+      <c r="C31" t="str">
+        <v>MTX#44 THEO_PHONG FULL</v>
+      </c>
+      <c r="D31" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E31" t="str">
+        <v>101</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Hồ Thị Long</v>
+      </c>
+      <c r="G31" t="str">
+        <v>079000000030</v>
+      </c>
+      <c r="H31" t="str">
+        <v>0904000030</v>
+      </c>
+      <c r="I31" t="str">
+        <v>1993-06-14</v>
+      </c>
+      <c r="J31" t="str">
+        <v>2023-06-24</v>
+      </c>
+      <c r="K31" t="str">
+        <v>CA Phú Nhuận</v>
+      </c>
+      <c r="L31" t="str">
+        <v>49 Lê Lợi, Quận 3</v>
+      </c>
+      <c r="M31" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="N31" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="O31">
+        <v>3300000</v>
+      </c>
+      <c r="P31">
+        <v>2</v>
+      </c>
+      <c r="Q31">
+        <v>6600000</v>
+      </c>
+      <c r="R31" t="str">
+        <v>2026-08-11</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>HD-MTX-45-RENO-RM-FULL</v>
+      </c>
+      <c r="B32" t="str">
+        <v/>
+      </c>
+      <c r="C32" t="str">
+        <v>MTX#45 THEO_PHONG FULL</v>
+      </c>
+      <c r="D32" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E32" t="str">
+        <v>101</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Nguyễn Thị Mai</v>
+      </c>
+      <c r="G32" t="str">
+        <v>079000000031</v>
+      </c>
+      <c r="H32" t="str">
+        <v>0904000031</v>
+      </c>
+      <c r="I32" t="str">
+        <v>1994-07-15</v>
+      </c>
+      <c r="J32" t="str">
+        <v>2018-07-10</v>
+      </c>
+      <c r="K32" t="str">
+        <v>CA TP. Hồ Chí Minh</v>
+      </c>
+      <c r="L32" t="str">
+        <v>50 Lê Lợi, Bình Thạnh</v>
+      </c>
+      <c r="M32" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="N32" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="O32">
+        <v>3700000</v>
+      </c>
+      <c r="P32">
+        <v>1</v>
+      </c>
+      <c r="Q32">
+        <v>3700000</v>
+      </c>
+      <c r="R32" t="str">
+        <v>2026-08-11</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>HD-MTX-46-RENO-RM-FULL</v>
+      </c>
+      <c r="B33" t="str">
+        <v/>
+      </c>
+      <c r="C33" t="str">
+        <v>MTX#46 THEO_PHONG FULL</v>
+      </c>
+      <c r="D33" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E33" t="str">
+        <v>101</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Trần Thị Nam</v>
+      </c>
+      <c r="G33" t="str">
+        <v>079000000032</v>
+      </c>
+      <c r="H33" t="str">
+        <v>0904000032</v>
+      </c>
+      <c r="I33" t="str">
+        <v>1995-08-16</v>
+      </c>
+      <c r="J33" t="str">
+        <v>2019-08-11</v>
+      </c>
+      <c r="K33" t="str">
+        <v>CA Quận 1</v>
+      </c>
+      <c r="L33" t="str">
+        <v>51 Lê Lợi, Gò Vấp</v>
+      </c>
+      <c r="M33" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="N33" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="O33">
+        <v>4100000</v>
+      </c>
+      <c r="P33">
+        <v>2</v>
+      </c>
+      <c r="Q33">
+        <v>8200000</v>
+      </c>
+      <c r="R33" t="str">
+        <v>2026-08-11</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>HD-MTX-47-RENO-RM-FULL</v>
+      </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v>MTX#47 THEO_PHONG FULL</v>
+      </c>
+      <c r="D34" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E34" t="str">
+        <v>101</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Lê Thị Oanh</v>
+      </c>
+      <c r="G34" t="str">
+        <v>079000000033</v>
+      </c>
+      <c r="H34" t="str">
+        <v>0904000033</v>
+      </c>
+      <c r="I34" t="str">
+        <v>1996-09-17</v>
+      </c>
+      <c r="J34" t="str">
+        <v>2020-09-12</v>
+      </c>
+      <c r="K34" t="str">
+        <v>CA Bình Thạnh</v>
+      </c>
+      <c r="L34" t="str">
+        <v>52 Lê Lợi, Phú Nhuận</v>
+      </c>
+      <c r="M34" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="N34" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="O34">
+        <v>4500000</v>
+      </c>
+      <c r="P34">
+        <v>1</v>
+      </c>
+      <c r="Q34">
+        <v>4500000</v>
+      </c>
+      <c r="R34" t="str">
+        <v>2026-08-11</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>HD-MTX-48-RENO-RM-HO-BUY</v>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v>MTX#48 THEO_PHONG BASIC</v>
+      </c>
+      <c r="D35" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E35" t="str">
+        <v>101</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Phạm Thị Phương</v>
+      </c>
+      <c r="G35" t="str">
+        <v>079000000034</v>
+      </c>
+      <c r="H35" t="str">
+        <v>0904000034</v>
+      </c>
+      <c r="I35" t="str">
+        <v>1997-10-18</v>
+      </c>
+      <c r="J35" t="str">
+        <v>2021-10-13</v>
+      </c>
+      <c r="K35" t="str">
+        <v>CA Gò Vấp</v>
+      </c>
+      <c r="L35" t="str">
+        <v>53 Lê Lợi, Cầu Giấy</v>
+      </c>
+      <c r="M35" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="N35" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="O35">
+        <v>2500000</v>
+      </c>
+      <c r="P35">
+        <v>2</v>
+      </c>
+      <c r="Q35">
+        <v>5000000</v>
+      </c>
+      <c r="R35" t="str">
+        <v>2026-08-11</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>HD-MTX-49-RENO-RM-HO-BUY</v>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v>MTX#49 THEO_PHONG BASIC</v>
+      </c>
+      <c r="D36" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E36" t="str">
+        <v>101</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Hoàng Thị Quân</v>
+      </c>
+      <c r="G36" t="str">
+        <v>079000000035</v>
+      </c>
+      <c r="H36" t="str">
+        <v>0904000035</v>
+      </c>
+      <c r="I36" t="str">
+        <v>1998-11-19</v>
+      </c>
+      <c r="J36" t="str">
+        <v>2022-11-14</v>
+      </c>
+      <c r="K36" t="str">
+        <v>CA Phú Nhuận</v>
+      </c>
+      <c r="L36" t="str">
+        <v>54 Lê Lợi, Quận 1</v>
+      </c>
+      <c r="M36" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="N36" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="O36">
+        <v>2900000</v>
+      </c>
+      <c r="P36">
+        <v>1</v>
+      </c>
+      <c r="Q36">
+        <v>2900000</v>
+      </c>
+      <c r="R36" t="str">
+        <v>2026-08-11</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>HD-MTX-50-RENO-RM-HO-BUY</v>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v>MTX#50 THEO_PHONG BASIC</v>
+      </c>
+      <c r="D37" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="E37" t="str">
+        <v>101</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Vũ Thị Quỳnh</v>
+      </c>
+      <c r="G37" t="str">
+        <v>079000000036</v>
+      </c>
+      <c r="H37" t="str">
+        <v>0904000036</v>
+      </c>
+      <c r="I37" t="str">
+        <v>1999-12-20</v>
+      </c>
+      <c r="J37" t="str">
+        <v>2023-12-15</v>
+      </c>
+      <c r="K37" t="str">
+        <v>CA TP. Hồ Chí Minh</v>
+      </c>
+      <c r="L37" t="str">
+        <v>55 Lê Lợi, Quận 3</v>
+      </c>
+      <c r="M37" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="N37" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="O37">
+        <v>3300000</v>
+      </c>
+      <c r="P37">
+        <v>2</v>
+      </c>
+      <c r="Q37">
+        <v>6600000</v>
+      </c>
+      <c r="R37" t="str">
+        <v>2026-08-11</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R37"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:M37"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2019,7 +2660,7 @@
     <col min="10" max="10" width="12.83203125" customWidth="1"/>
     <col min="11" max="11" width="12.83203125" customWidth="1"/>
     <col min="12" max="12" width="36.83203125" customWidth="1"/>
-    <col min="13" max="13" width="36.83203125" customWidth="1"/>
+    <col min="13" max="13" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2921,7 +3562,7 @@
         <v>REJECT confirm 11/08 (sớm 5 ngày)</v>
       </c>
       <c r="M22" t="str">
-        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101</v>
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (không nội thất)</v>
       </c>
     </row>
     <row r="23">
@@ -2962,7 +3603,7 @@
         <v>REJECT confirm 11/08 (sớm 7 ngày)</v>
       </c>
       <c r="M23" t="str">
-        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101</v>
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (không nội thất)</v>
       </c>
     </row>
     <row r="24">
@@ -3003,7 +3644,7 @@
         <v>REJECT confirm 11/08 (sớm 9 ngày)</v>
       </c>
       <c r="M24" t="str">
-        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101</v>
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (không nội thất)</v>
       </c>
     </row>
     <row r="25">
@@ -3044,7 +3685,7 @@
         <v>REJECT confirm 11/08 (sớm 14 ngày)</v>
       </c>
       <c r="M25" t="str">
-        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101</v>
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (không nội thất)</v>
       </c>
     </row>
     <row r="26">
@@ -3085,12 +3726,463 @@
         <v>REJECT confirm 11/08 (sớm ~3 tuần)</v>
       </c>
       <c r="M26" t="str">
-        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101</v>
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (nội thất cơ bản)</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>D1</v>
+      </c>
+      <c r="C27" t="str">
+        <v>MTX40+</v>
+      </c>
+      <c r="D27" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E27" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F27" t="str">
+        <v>HD-MTX-40-RENO-RM-BASIC-BUY</v>
+      </c>
+      <c r="G27" t="str">
+        <v>MTX#40 THEO_PHONG BASIC</v>
+      </c>
+      <c r="H27" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="I27" t="str">
+        <v>101</v>
+      </c>
+      <c r="J27" t="str">
+        <v>tenant26</v>
+      </c>
+      <c r="K27" t="str">
+        <v>0904000026</v>
+      </c>
+      <c r="L27" t="str">
+        <v>OK confirm 11/08 — MTX#40</v>
+      </c>
+      <c r="M27" t="str">
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (nội thất cơ bản)</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>D2</v>
+      </c>
+      <c r="C28" t="str">
+        <v>MTX40+</v>
+      </c>
+      <c r="D28" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E28" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F28" t="str">
+        <v>HD-MTX-41-RENO-RM-BASIC-BUY</v>
+      </c>
+      <c r="G28" t="str">
+        <v>MTX#41 THEO_PHONG BASIC</v>
+      </c>
+      <c r="H28" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="I28" t="str">
+        <v>101</v>
+      </c>
+      <c r="J28" t="str">
+        <v>tenant27</v>
+      </c>
+      <c r="K28" t="str">
+        <v>0904000027</v>
+      </c>
+      <c r="L28" t="str">
+        <v>OK confirm 11/08 — MTX#41</v>
+      </c>
+      <c r="M28" t="str">
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (nội thất cơ bản)</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>D3</v>
+      </c>
+      <c r="C29" t="str">
+        <v>MTX40+</v>
+      </c>
+      <c r="D29" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E29" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F29" t="str">
+        <v>HD-MTX-42-RENO-RM-BASIC-BUY</v>
+      </c>
+      <c r="G29" t="str">
+        <v>MTX#42 THEO_PHONG BASIC</v>
+      </c>
+      <c r="H29" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="I29" t="str">
+        <v>101</v>
+      </c>
+      <c r="J29" t="str">
+        <v>tenant28</v>
+      </c>
+      <c r="K29" t="str">
+        <v>0904000028</v>
+      </c>
+      <c r="L29" t="str">
+        <v>OK confirm 11/08 — MTX#42</v>
+      </c>
+      <c r="M29" t="str">
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (nội thất cơ bản)</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>D4</v>
+      </c>
+      <c r="C30" t="str">
+        <v>MTX40+</v>
+      </c>
+      <c r="D30" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E30" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F30" t="str">
+        <v>HD-MTX-43-RENO-RM-BASIC-BUY</v>
+      </c>
+      <c r="G30" t="str">
+        <v>MTX#43 THEO_PHONG BASIC</v>
+      </c>
+      <c r="H30" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="I30" t="str">
+        <v>101</v>
+      </c>
+      <c r="J30" t="str">
+        <v>tenant29</v>
+      </c>
+      <c r="K30" t="str">
+        <v>0904000029</v>
+      </c>
+      <c r="L30" t="str">
+        <v>OK confirm 11/08 — MTX#43</v>
+      </c>
+      <c r="M30" t="str">
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (nội thất cơ bản)</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>D5</v>
+      </c>
+      <c r="C31" t="str">
+        <v>MTX40+</v>
+      </c>
+      <c r="D31" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E31" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F31" t="str">
+        <v>HD-MTX-44-RENO-RM-FULL</v>
+      </c>
+      <c r="G31" t="str">
+        <v>MTX#44 THEO_PHONG FULL</v>
+      </c>
+      <c r="H31" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="I31" t="str">
+        <v>101</v>
+      </c>
+      <c r="J31" t="str">
+        <v>tenant30</v>
+      </c>
+      <c r="K31" t="str">
+        <v>0904000030</v>
+      </c>
+      <c r="L31" t="str">
+        <v>OK confirm 11/08 — MTX#44</v>
+      </c>
+      <c r="M31" t="str">
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (full nội thất)</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>D6</v>
+      </c>
+      <c r="C32" t="str">
+        <v>MTX40+</v>
+      </c>
+      <c r="D32" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E32" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F32" t="str">
+        <v>HD-MTX-45-RENO-RM-FULL</v>
+      </c>
+      <c r="G32" t="str">
+        <v>MTX#45 THEO_PHONG FULL</v>
+      </c>
+      <c r="H32" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="I32" t="str">
+        <v>101</v>
+      </c>
+      <c r="J32" t="str">
+        <v>tenant31</v>
+      </c>
+      <c r="K32" t="str">
+        <v>0904000031</v>
+      </c>
+      <c r="L32" t="str">
+        <v>OK confirm 11/08 — MTX#45</v>
+      </c>
+      <c r="M32" t="str">
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (full nội thất)</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>D7</v>
+      </c>
+      <c r="C33" t="str">
+        <v>MTX40+</v>
+      </c>
+      <c r="D33" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E33" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F33" t="str">
+        <v>HD-MTX-46-RENO-RM-FULL</v>
+      </c>
+      <c r="G33" t="str">
+        <v>MTX#46 THEO_PHONG FULL</v>
+      </c>
+      <c r="H33" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="I33" t="str">
+        <v>101</v>
+      </c>
+      <c r="J33" t="str">
+        <v>tenant32</v>
+      </c>
+      <c r="K33" t="str">
+        <v>0904000032</v>
+      </c>
+      <c r="L33" t="str">
+        <v>OK confirm 11/08 — MTX#46</v>
+      </c>
+      <c r="M33" t="str">
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (full nội thất)</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>D8</v>
+      </c>
+      <c r="C34" t="str">
+        <v>MTX40+</v>
+      </c>
+      <c r="D34" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E34" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F34" t="str">
+        <v>HD-MTX-47-RENO-RM-FULL</v>
+      </c>
+      <c r="G34" t="str">
+        <v>MTX#47 THEO_PHONG FULL</v>
+      </c>
+      <c r="H34" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="I34" t="str">
+        <v>101</v>
+      </c>
+      <c r="J34" t="str">
+        <v>tenant33</v>
+      </c>
+      <c r="K34" t="str">
+        <v>0904000033</v>
+      </c>
+      <c r="L34" t="str">
+        <v>OK confirm 11/08 — MTX#47</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (full nội thất)</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>D9</v>
+      </c>
+      <c r="C35" t="str">
+        <v>MTX40+</v>
+      </c>
+      <c r="D35" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E35" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F35" t="str">
+        <v>HD-MTX-48-RENO-RM-HO-BUY</v>
+      </c>
+      <c r="G35" t="str">
+        <v>MTX#48 THEO_PHONG BASIC</v>
+      </c>
+      <c r="H35" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="I35" t="str">
+        <v>101</v>
+      </c>
+      <c r="J35" t="str">
+        <v>tenant34</v>
+      </c>
+      <c r="K35" t="str">
+        <v>0904000034</v>
+      </c>
+      <c r="L35" t="str">
+        <v>OK confirm 11/08 — MTX#48</v>
+      </c>
+      <c r="M35" t="str">
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (nội thất cơ bản)</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>D10</v>
+      </c>
+      <c r="C36" t="str">
+        <v>MTX40+</v>
+      </c>
+      <c r="D36" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E36" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F36" t="str">
+        <v>HD-MTX-49-RENO-RM-HO-BUY</v>
+      </c>
+      <c r="G36" t="str">
+        <v>MTX#49 THEO_PHONG BASIC</v>
+      </c>
+      <c r="H36" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="I36" t="str">
+        <v>101</v>
+      </c>
+      <c r="J36" t="str">
+        <v>tenant35</v>
+      </c>
+      <c r="K36" t="str">
+        <v>0904000035</v>
+      </c>
+      <c r="L36" t="str">
+        <v>OK confirm 11/08 — MTX#49</v>
+      </c>
+      <c r="M36" t="str">
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (nội thất cơ bản)</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>D11</v>
+      </c>
+      <c r="C37" t="str">
+        <v>MTX40+</v>
+      </c>
+      <c r="D37" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="E37" t="str">
+        <v>2027-08-10</v>
+      </c>
+      <c r="F37" t="str">
+        <v>HD-MTX-50-RENO-RM-HO-BUY</v>
+      </c>
+      <c r="G37" t="str">
+        <v>MTX#50 THEO_PHONG BASIC</v>
+      </c>
+      <c r="H37" t="str">
+        <v>THEO_PHONG</v>
+      </c>
+      <c r="I37" t="str">
+        <v>101</v>
+      </c>
+      <c r="J37" t="str">
+        <v>tenant36</v>
+      </c>
+      <c r="K37" t="str">
+        <v>0904000036</v>
+      </c>
+      <c r="L37" t="str">
+        <v>OK confirm 11/08 — MTX#50</v>
+      </c>
+      <c r="M37" t="str">
+        <v>Cần import đợt 2 (THEO_PHONG) trước — phòng 101 (nội thất cơ bản)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>